<commit_message>
update: Attendance Report add Start/End Working date
</commit_message>
<xml_diff>
--- a/server/templates/attendance-report-template.xlsx
+++ b/server/templates/attendance-report-template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Asus\Documents\projects\nanafruit-hrm\server\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E1658796-D567-4429-A977-B00BB2A1ACA9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DCDE42A4-5694-4283-94E3-D54F1FA1C12F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="24">
   <si>
     <t>รายงานการลงเวลา ตั้งแต่วันที่ 26/07/2026 ถึง 25/08/2026</t>
   </si>
@@ -102,6 +102,12 @@
   </si>
   <si>
     <t xml:space="preserve"> 08:30-17:30</t>
+  </si>
+  <si>
+    <t>วันที่เริ่มงาน</t>
+  </si>
+  <si>
+    <t>วันที่สิ้นสุดการทำงาน</t>
   </si>
 </sst>
 </file>
@@ -545,23 +551,25 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K3"/>
+  <dimension ref="A1:M3"/>
   <sheetFormatPr defaultRowHeight="17.25" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="16.85546875" style="1" customWidth="1"/>
     <col min="2" max="2" width="31" style="1" customWidth="1"/>
-    <col min="3" max="3" width="26" style="1" customWidth="1"/>
-    <col min="4" max="4" width="20.42578125" style="1" customWidth="1"/>
-    <col min="5" max="5" width="26.5703125" style="1" customWidth="1"/>
-    <col min="6" max="6" width="18.5703125" style="1" customWidth="1"/>
-    <col min="7" max="8" width="19.42578125" style="1" customWidth="1"/>
-    <col min="9" max="9" width="21.42578125" style="1" customWidth="1"/>
-    <col min="10" max="10" width="20.7109375" style="1" customWidth="1"/>
-    <col min="11" max="11" width="22.7109375" style="1" customWidth="1"/>
-    <col min="12" max="16384" width="9.140625" style="1"/>
+    <col min="3" max="3" width="22.85546875" style="1" customWidth="1"/>
+    <col min="4" max="4" width="21.28515625" style="1" customWidth="1"/>
+    <col min="5" max="5" width="26" style="1" customWidth="1"/>
+    <col min="6" max="6" width="20.42578125" style="1" customWidth="1"/>
+    <col min="7" max="7" width="26.5703125" style="1" customWidth="1"/>
+    <col min="8" max="8" width="18.5703125" style="1" customWidth="1"/>
+    <col min="9" max="10" width="19.42578125" style="1" customWidth="1"/>
+    <col min="11" max="11" width="21.42578125" style="1" customWidth="1"/>
+    <col min="12" max="12" width="20.7109375" style="1" customWidth="1"/>
+    <col min="13" max="13" width="22.7109375" style="1" customWidth="1"/>
+    <col min="14" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="31.5" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:13" ht="31.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
@@ -575,8 +583,10 @@
       <c r="I1" s="5"/>
       <c r="J1" s="5"/>
       <c r="K1" s="5"/>
+      <c r="L1" s="5"/>
+      <c r="M1" s="5"/>
     </row>
-    <row r="2" spans="1:11" s="2" customFormat="1" ht="24" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:13" s="2" customFormat="1" ht="24" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
         <v>1</v>
       </c>
@@ -584,65 +594,77 @@
         <v>2</v>
       </c>
       <c r="C2" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="D2" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="E2" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="D2" s="6" t="s">
+      <c r="F2" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="E2" s="6" t="s">
+      <c r="G2" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="F2" s="6" t="s">
+      <c r="H2" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="G2" s="6" t="s">
+      <c r="I2" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="H2" s="6" t="s">
+      <c r="J2" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="I2" s="6" t="s">
+      <c r="K2" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="J2" s="6" t="s">
+      <c r="L2" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="K2" s="6" t="s">
+      <c r="M2" s="6" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:11" s="3" customFormat="1" ht="24" x14ac:dyDescent="0.55000000000000004">
+    <row r="3" spans="1:13" s="3" customFormat="1" ht="24" x14ac:dyDescent="0.55000000000000004">
       <c r="A3" s="7" t="s">
         <v>11</v>
       </c>
       <c r="B3" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="C3" s="8" t="s">
+      <c r="C3" s="9">
+        <v>46244</v>
+      </c>
+      <c r="D3" s="9">
+        <v>2958465</v>
+      </c>
+      <c r="E3" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="D3" s="8" t="s">
+      <c r="F3" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="E3" s="7" t="s">
+      <c r="G3" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="F3" s="9">
+      <c r="H3" s="9">
         <v>46253</v>
       </c>
-      <c r="G3" s="7" t="s">
+      <c r="I3" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="H3" s="7" t="s">
+      <c r="J3" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="I3" s="7" t="s">
+      <c r="K3" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="J3" s="10" t="s">
+      <c r="L3" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="K3" s="8" t="s">
+      <c r="M3" s="8" t="s">
         <v>18</v>
       </c>
     </row>

</xml_diff>

<commit_message>
update: Daily Temporary Employee import and Shift assignment
</commit_message>
<xml_diff>
--- a/server/templates/attendance-report-template.xlsx
+++ b/server/templates/attendance-report-template.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Asus\Documents\projects\nanafruit-hrm\server\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DCDE42A4-5694-4283-94E3-D54F1FA1C12F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B3458FF2-E83A-411C-A44C-9D4915A0254E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -165,12 +165,18 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="3">
@@ -224,9 +230,6 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -236,6 +239,9 @@
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -587,84 +593,84 @@
       <c r="M1" s="5"/>
     </row>
     <row r="2" spans="1:13" s="2" customFormat="1" ht="24" x14ac:dyDescent="0.25">
-      <c r="A2" s="6" t="s">
+      <c r="A2" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="6" t="s">
+      <c r="B2" s="10" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="6" t="s">
+      <c r="C2" s="10" t="s">
         <v>22</v>
       </c>
-      <c r="D2" s="6" t="s">
+      <c r="D2" s="10" t="s">
         <v>23</v>
       </c>
-      <c r="E2" s="6" t="s">
+      <c r="E2" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="F2" s="6" t="s">
+      <c r="F2" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="G2" s="6" t="s">
+      <c r="G2" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="H2" s="6" t="s">
+      <c r="H2" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="I2" s="6" t="s">
+      <c r="I2" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="J2" s="6" t="s">
+      <c r="J2" s="10" t="s">
         <v>20</v>
       </c>
-      <c r="K2" s="6" t="s">
+      <c r="K2" s="10" t="s">
         <v>8</v>
       </c>
-      <c r="L2" s="6" t="s">
+      <c r="L2" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="M2" s="6" t="s">
+      <c r="M2" s="10" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="3" spans="1:13" s="3" customFormat="1" ht="24" x14ac:dyDescent="0.55000000000000004">
-      <c r="A3" s="7" t="s">
+      <c r="A3" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="B3" s="8" t="s">
+      <c r="B3" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="C3" s="9">
+      <c r="C3" s="8">
         <v>46244</v>
       </c>
-      <c r="D3" s="9">
+      <c r="D3" s="8">
         <v>2958465</v>
       </c>
-      <c r="E3" s="8" t="s">
+      <c r="E3" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="F3" s="8" t="s">
+      <c r="F3" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="G3" s="7" t="s">
+      <c r="G3" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="H3" s="9">
+      <c r="H3" s="8">
         <v>46253</v>
       </c>
-      <c r="I3" s="7" t="s">
+      <c r="I3" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="J3" s="7" t="s">
+      <c r="J3" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="K3" s="7" t="s">
+      <c r="K3" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="L3" s="10" t="s">
+      <c r="L3" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="M3" s="8" t="s">
+      <c r="M3" s="7" t="s">
         <v>18</v>
       </c>
     </row>

</xml_diff>

<commit_message>
update: Add Fingerprint Code on Attendance Report
</commit_message>
<xml_diff>
--- a/server/templates/attendance-report-template.xlsx
+++ b/server/templates/attendance-report-template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Asus\Documents\projects\nanafruit-hrm\server\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B3458FF2-E83A-411C-A44C-9D4915A0254E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FC8ED709-1FD4-4980-98D1-B50271B51DE9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="26">
   <si>
     <t>รายงานการลงเวลา ตั้งแต่วันที่ 26/07/2026 ถึง 25/08/2026</t>
   </si>
@@ -108,6 +108,12 @@
   </si>
   <si>
     <t>วันที่สิ้นสุดการทำงาน</t>
+  </si>
+  <si>
+    <t>รหัสลายนิ้วมือ</t>
+  </si>
+  <si>
+    <t>FP9999</t>
   </si>
 </sst>
 </file>
@@ -557,29 +563,29 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:M3"/>
+  <dimension ref="A1:N3"/>
   <sheetFormatPr defaultRowHeight="17.25" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="16.85546875" style="1" customWidth="1"/>
-    <col min="2" max="2" width="31" style="1" customWidth="1"/>
-    <col min="3" max="3" width="22.85546875" style="1" customWidth="1"/>
-    <col min="4" max="4" width="21.28515625" style="1" customWidth="1"/>
-    <col min="5" max="5" width="26" style="1" customWidth="1"/>
-    <col min="6" max="6" width="20.42578125" style="1" customWidth="1"/>
-    <col min="7" max="7" width="26.5703125" style="1" customWidth="1"/>
-    <col min="8" max="8" width="18.5703125" style="1" customWidth="1"/>
-    <col min="9" max="10" width="19.42578125" style="1" customWidth="1"/>
-    <col min="11" max="11" width="21.42578125" style="1" customWidth="1"/>
-    <col min="12" max="12" width="20.7109375" style="1" customWidth="1"/>
-    <col min="13" max="13" width="22.7109375" style="1" customWidth="1"/>
-    <col min="14" max="16384" width="9.140625" style="1"/>
+    <col min="1" max="2" width="16.85546875" style="1" customWidth="1"/>
+    <col min="3" max="3" width="31" style="1" customWidth="1"/>
+    <col min="4" max="4" width="22.85546875" style="1" customWidth="1"/>
+    <col min="5" max="5" width="21.28515625" style="1" customWidth="1"/>
+    <col min="6" max="6" width="26" style="1" customWidth="1"/>
+    <col min="7" max="7" width="20.42578125" style="1" customWidth="1"/>
+    <col min="8" max="8" width="26.5703125" style="1" customWidth="1"/>
+    <col min="9" max="9" width="18.5703125" style="1" customWidth="1"/>
+    <col min="10" max="11" width="19.42578125" style="1" customWidth="1"/>
+    <col min="12" max="12" width="21.42578125" style="1" customWidth="1"/>
+    <col min="13" max="13" width="20.7109375" style="1" customWidth="1"/>
+    <col min="14" max="14" width="22.7109375" style="1" customWidth="1"/>
+    <col min="15" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" ht="31.5" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:14" ht="31.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="5"/>
+      <c r="B1" s="4"/>
       <c r="C1" s="5"/>
       <c r="D1" s="5"/>
       <c r="E1" s="5"/>
@@ -591,86 +597,93 @@
       <c r="K1" s="5"/>
       <c r="L1" s="5"/>
       <c r="M1" s="5"/>
+      <c r="N1" s="5"/>
     </row>
-    <row r="2" spans="1:13" s="2" customFormat="1" ht="24" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:14" s="2" customFormat="1" ht="24" x14ac:dyDescent="0.25">
       <c r="A2" s="10" t="s">
         <v>1</v>
       </c>
       <c r="B2" s="10" t="s">
+        <v>24</v>
+      </c>
+      <c r="C2" s="10" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="10" t="s">
+      <c r="D2" s="10" t="s">
         <v>22</v>
       </c>
-      <c r="D2" s="10" t="s">
+      <c r="E2" s="10" t="s">
         <v>23</v>
       </c>
-      <c r="E2" s="10" t="s">
+      <c r="F2" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="F2" s="10" t="s">
+      <c r="G2" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="G2" s="10" t="s">
+      <c r="H2" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="H2" s="10" t="s">
+      <c r="I2" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="I2" s="10" t="s">
+      <c r="J2" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="J2" s="10" t="s">
+      <c r="K2" s="10" t="s">
         <v>20</v>
       </c>
-      <c r="K2" s="10" t="s">
+      <c r="L2" s="10" t="s">
         <v>8</v>
       </c>
-      <c r="L2" s="10" t="s">
+      <c r="M2" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="M2" s="10" t="s">
+      <c r="N2" s="10" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:13" s="3" customFormat="1" ht="24" x14ac:dyDescent="0.55000000000000004">
+    <row r="3" spans="1:14" s="3" customFormat="1" ht="24" x14ac:dyDescent="0.55000000000000004">
       <c r="A3" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="B3" s="7" t="s">
+      <c r="B3" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="C3" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="C3" s="8">
+      <c r="D3" s="8">
         <v>46244</v>
       </c>
-      <c r="D3" s="8">
+      <c r="E3" s="8">
         <v>2958465</v>
       </c>
-      <c r="E3" s="7" t="s">
+      <c r="F3" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="F3" s="7" t="s">
+      <c r="G3" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="G3" s="6" t="s">
+      <c r="H3" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="H3" s="8">
+      <c r="I3" s="8">
         <v>46253</v>
       </c>
-      <c r="I3" s="6" t="s">
+      <c r="J3" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="J3" s="6" t="s">
+      <c r="K3" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="K3" s="6" t="s">
+      <c r="L3" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="L3" s="9" t="s">
+      <c r="M3" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="M3" s="7" t="s">
+      <c r="N3" s="7" t="s">
         <v>18</v>
       </c>
     </row>

</xml_diff>